<commit_message>
import to google calendar
</commit_message>
<xml_diff>
--- a/my_studysmart.xlsx
+++ b/my_studysmart.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,18 +453,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>stats</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D2" t="inlineStr"/>
+        <v>35</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Chapter 1, Chapter 2, Chapter 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Neuro</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>30</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>M, W, E, R</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>